<commit_message>
feat: enforce unique major codes and refine graduation filters
</commit_message>
<xml_diff>
--- a/docs/import-data/danh-sach-nganh-dao-tao-day-du.xlsx
+++ b/docs/import-data/danh-sach-nganh-dao-tao-day-du.xlsx
@@ -273,34 +273,64 @@
     <t>Máy và tự động hóa xếp dỡ</t>
   </si>
   <si>
+    <t>CNT-CLC</t>
+  </si>
+  <si>
     <t>Công nghệ thông tin (CLC)</t>
   </si>
   <si>
     <t>Viện Đào tạo chất lượng cao</t>
   </si>
   <si>
+    <t>CNT-NC</t>
+  </si>
+  <si>
     <t>Công nghệ thông tin (NC)</t>
   </si>
   <si>
+    <t>ĐTĐ-CLC</t>
+  </si>
+  <si>
     <t>Điện tự động công nghiệp (CLC)</t>
   </si>
   <si>
+    <t>ĐTĐ-NC</t>
+  </si>
+  <si>
     <t>Điện tự động công nghiệp (NC)</t>
   </si>
   <si>
+    <t>ĐKT-C</t>
+  </si>
+  <si>
     <t>Điều khiển tàu biển (Chọn)</t>
   </si>
   <si>
+    <t>MKT-C</t>
+  </si>
+  <si>
     <t>Khai thác máy tàu biển (Chọn)</t>
   </si>
   <si>
+    <t>KTN-CLC</t>
+  </si>
+  <si>
     <t>Kinh tế ngoại thương (CLC)</t>
   </si>
   <si>
+    <t>KTN-NC</t>
+  </si>
+  <si>
     <t>Kinh tế ngoại thương (NC)</t>
   </si>
   <si>
+    <t>KTB-CLC</t>
+  </si>
+  <si>
     <t>Kinh tế vận tải biển (CLC)</t>
+  </si>
+  <si>
+    <t>KTB-NC</t>
   </si>
   <si>
     <t>Kinh tế vận tải biển (NC)</t>
@@ -860,167 +890,167 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C38" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>6</v>
+        <v>88</v>
       </c>
       <c r="B39" t="s">
+        <v>89</v>
+      </c>
+      <c r="C39" t="s">
         <v>87</v>
-      </c>
-      <c r="C39" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="B40" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>37</v>
+        <v>94</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>96</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C43" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>98</v>
       </c>
       <c r="B44" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C44" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>100</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C45" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>102</v>
       </c>
       <c r="B46" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C46" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="C47" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="C48" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="B49" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="C49" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="B50" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="B51" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="C51" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B52" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C52" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1035,12 +1065,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3">
@@ -1055,7 +1085,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -1070,7 +1100,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9">
@@ -1100,17 +1130,17 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17">
@@ -1120,17 +1150,17 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1145,32 +1175,32 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>